<commit_message>
docs & test: finalize unit test suite, CSV tests, Excel specs, and documentation
</commit_message>
<xml_diff>
--- a/documents/Test_Cases_Specification.xlsx
+++ b/documents/Test_Cases_Specification.xlsx
@@ -9,8 +9,7 @@
   <sheets>
     <sheet name="Email Validation" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="IP Address Validation" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="URL Validation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="CSV External Data Tests" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CSV External Data Tests" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2350,825 +2349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="51" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Test ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Module</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Function</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Test Input</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Expected Output</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Technique</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>TC-URL-01</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>validators.url</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>https://google.com</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>True (Valid)</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>ECP</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Smoke/ECP</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>TC-URL-02</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>validators.url</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>http://example.org</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>True (Valid)</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>ECP</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>ECP</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>TC-URL-03</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>validators.url</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>ftp://files.example.com</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>True (Valid)</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>ECP</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>ECP</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>TC-URL-04</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>validators.url</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>https://fast.edu.pk:8080</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>True (Valid)</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>ECP</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>ECP</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>TC-URL-05</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>validators.url</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>https://example.com/api/v1?search=test&amp;sort=asc</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>True (Valid)</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>ECP</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>ECP</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>TC-URL-06</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>validators.url</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>https://example.com/home#section2</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>True (Valid)</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>ECP</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>ECP</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>TC-URL-07</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>validators.url</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>not-a-url</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>False (Invalid)</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>ECP</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>ECP/Regression</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>TC-URL-08</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>validators.url</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>htp://wrong-scheme.com</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>False (Invalid)</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>ECP</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>ECP/Regression</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>TC-URL-09</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>validators.url</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>http://</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>False (Invalid)</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>ECP</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>ECP/Regression</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>TC-URL-10</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>validators.url</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>https://exam ple.com</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>False (Invalid)</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>ECP</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>ECP/Regression</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>TC-URL-11</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>validators.url</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>javascript:alert(1)</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>False (Invalid)</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>ECP</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>ECP/Regression</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>TC-URL-12</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>validators.url</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>http://-leading-hyphen.com</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>False (Invalid)</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>ECP</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>ECP/Regression</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>TC-URL-13</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>validators.url</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>http://a.io</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>True (Valid)</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>BVA</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>BVA/Regression</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>TC-URL-14</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>validators.url</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>http://example.com:1</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>True (Valid)</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>BVA</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>BVA/Regression</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>TC-URL-15</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>validators.url</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>http://example.com:65535</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>True (Valid)</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>BVA</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>BVA/Regression</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>TC-URL-16</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>validators.url</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>http://example.com:65536</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>False (Invalid)</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>BVA</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>BVA/Regression</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>TC-URL-17</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>validators.url</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>http://example.com:0</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>False (Invalid)</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>BVA</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>BVA/Regression</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>TC-URL-18</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>validators.url</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>False (Invalid)</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>BVA</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>BVA/Regression</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3478,37 +2659,37 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>I-01</t>
+          <t>E-07</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>ip_data.csv</t>
+          <t>email_data.csv</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>validators.ipv4</t>
+          <t>validators.email</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>192.168.1.1</t>
+          <t>a@b.c</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>invalid</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>ECP</t>
+          <t>BVA</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>CSV/IP</t>
+          <t>CSV/Email</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -3520,7 +2701,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>I-02</t>
+          <t>I-01</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -3535,17 +2716,17 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>256.1.1.1</t>
+          <t>192.168.1.1</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>BVA</t>
+          <t>ECP</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -3562,7 +2743,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>I-03</t>
+          <t>I-02</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -3577,7 +2758,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>1.2.3</t>
+          <t>256.1.1.1</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -3587,7 +2768,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>ECP</t>
+          <t>BVA</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -3604,7 +2785,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>I-04</t>
+          <t>I-03</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -3614,17 +2795,17 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>validators.ipv6</t>
+          <t>validators.ipv4</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>::1</t>
+          <t>1.2.3</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -3646,7 +2827,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>I-05</t>
+          <t>I-04</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -3661,17 +2842,17 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>1:2:3:4:5:6:7:8:9</t>
+          <t>::1</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>FALSE</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>BVA</t>
+          <t>ECP</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -3688,40 +2869,82 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>I-05</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>ip_data.csv</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>validators.ipv6</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>1:2:3:4:5:6:7:8:9</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>BVA</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>CSV/IP</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>I-06</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>ip_data.csv</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>validators.ipv6</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>gggg::1</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>ECP</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>ECP</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>CSV/IP</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>

</xml_diff>